<commit_message>
mappatura NoiPA corretto script per dataset con formato URL diverso
</commit_message>
<xml_diff>
--- a/mappatura_noipa.xlsx
+++ b/mappatura_noipa.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t xml:space="preserve">Dati stipendi NoiPA - dataset</t>
   </si>
@@ -198,6 +198,18 @@
   </si>
   <si>
     <t xml:space="preserve">n_obs=8869; n_col=8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Redditi di lavoro dipendente e assimilati certificati agli Amministrati</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">amministrazione|eta_min|eta_max|sesso|anno|regione_di_residenza|imponibili_previdenziali|reddito_relativo_anno_corrente|reddito_relativo_anni_precedenti|ritenute_comunali|ritenute_regionali|ritenute_irpef_anno_corrente|ritenute_irpef_anno_precedente|totale_detrazioni|previdenza_complementare|numero_amministrati</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_obs=4053; n_col=16</t>
   </si>
   <si>
     <t xml:space="preserve">Amministrati per Fascia di Reddito</t>
@@ -554,10 +566,10 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="50.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="71.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="30.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="32.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="136.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="250.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="32.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="27.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="20.71" hidden="0" customWidth="1"/>
@@ -969,11 +981,11 @@
         <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>9</v>
+        <v>63</v>
       </c>
       <c r="C19"/>
       <c r="D19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E19" t="s">
         <v>11</v>
@@ -983,7 +995,29 @@
         <v>12</v>
       </c>
       <c r="H19" t="s">
-        <v>64</v>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20"/>
+      <c r="D20" t="s">
+        <v>67</v>
+      </c>
+      <c r="E20" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20"/>
+      <c r="G20" t="s">
+        <v>12</v>
+      </c>
+      <c r="H20" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>